<commit_message>
Experiment 4: Add sw (water saturation) as 6th feature, optimize blend alpha to 0.55
Subsurface feature sweep showed sw improves both C-index (0.821→0.858) and
MAE (58→50 months) via LOOCV. All other subsurface features (porosity,
permeability, dist_to_gwc, net_pay, chlorides, perf_thickness) degraded or
were neutral. Updated vertical and horizontal prediction notebooks, figures,
results, and documentation.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mari_poc/horizontal_predictions/results/horizontal_predictions.xlsx
+++ b/mari_poc/horizontal_predictions/results/horizontal_predictions.xlsx
@@ -504,19 +504,19 @@
         <v>25</v>
       </c>
       <c r="F2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G2" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H2" t="n">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="I2" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="J2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -537,22 +537,22 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="F3" t="n">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="G3" t="n">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="H3" t="n">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="I3" t="n">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="J3" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
@@ -570,25 +570,25 @@
         <v>18</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="E4" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F4" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G4" t="n">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="H4" t="n">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="I4" t="n">
-        <v>305</v>
+        <v>289</v>
       </c>
       <c r="J4" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5">
@@ -606,25 +606,25 @@
         <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="F5" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="G5" t="n">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="H5" t="n">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="I5" t="n">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="J5" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -642,25 +642,25 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E6" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F6" t="n">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="G6" t="n">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="H6" t="n">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="I6" t="n">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="J6" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -744,7 +744,7 @@
         <v>45</v>
       </c>
       <c r="C2" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -753,13 +753,13 @@
         <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="G2" t="n">
         <v>169</v>
       </c>
       <c r="H2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I2" t="n">
         <v>71</v>
@@ -768,7 +768,7 @@
         <v>84</v>
       </c>
       <c r="K2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3">
@@ -781,22 +781,22 @@
         <v>45</v>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>42</v>
       </c>
       <c r="F3" t="n">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="G3" t="n">
         <v>307</v>
       </c>
       <c r="H3" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I3" t="n">
         <v>114</v>
@@ -805,7 +805,7 @@
         <v>200</v>
       </c>
       <c r="K3" t="n">
-        <v>153</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4">
@@ -818,31 +818,31 @@
         <v>45</v>
       </c>
       <c r="C4" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>42</v>
       </c>
       <c r="F4" t="n">
-        <v>219</v>
+        <v>194</v>
       </c>
       <c r="G4" t="n">
         <v>242</v>
       </c>
       <c r="H4" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I4" t="n">
         <v>101</v>
       </c>
       <c r="J4" t="n">
-        <v>226</v>
+        <v>200</v>
       </c>
       <c r="K4" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5">
@@ -855,22 +855,22 @@
         <v>45</v>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>42</v>
       </c>
       <c r="F5" t="n">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="G5" t="n">
         <v>181</v>
       </c>
       <c r="H5" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I5" t="n">
         <v>88</v>
@@ -879,7 +879,7 @@
         <v>174</v>
       </c>
       <c r="K5" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6">
@@ -892,7 +892,7 @@
         <v>45</v>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -901,13 +901,13 @@
         <v>30</v>
       </c>
       <c r="F6" t="n">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="G6" t="n">
         <v>147</v>
       </c>
       <c r="H6" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I6" t="n">
         <v>67</v>
@@ -916,7 +916,7 @@
         <v>148</v>
       </c>
       <c r="K6" t="n">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -991,10 +991,20 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>sw (raw)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>sw (scaled)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>peak_gas_rate_raw</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>perf_thickness_m</t>
         </is>
@@ -1037,9 +1047,15 @@
         <v>0.008</v>
       </c>
       <c r="L2" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="n">
         <v>409</v>
       </c>
-      <c r="M2" t="n">
+      <c r="O2" t="n">
         <v>530</v>
       </c>
     </row>
@@ -1080,9 +1096,15 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.515</v>
+      </c>
+      <c r="N3" t="n">
         <v>300</v>
       </c>
-      <c r="M3" t="n">
+      <c r="O3" t="n">
         <v>802</v>
       </c>
     </row>
@@ -1123,9 +1145,15 @@
         <v>0.013</v>
       </c>
       <c r="L4" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
         <v>476</v>
       </c>
-      <c r="M4" t="n">
+      <c r="O4" t="n">
         <v>475</v>
       </c>
     </row>
@@ -1166,9 +1194,15 @@
         <v>0.001</v>
       </c>
       <c r="L5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.515</v>
+      </c>
+      <c r="N5" t="n">
         <v>334</v>
       </c>
-      <c r="M5" t="n">
+      <c r="O5" t="n">
         <v>758</v>
       </c>
     </row>
@@ -1209,9 +1243,15 @@
         <v>0.001</v>
       </c>
       <c r="L6" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="n">
         <v>298</v>
       </c>
-      <c r="M6" t="n">
+      <c r="O6" t="n">
         <v>719</v>
       </c>
     </row>
@@ -1304,13 +1344,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1.646</v>
+        <v>1.638</v>
       </c>
       <c r="H2" t="n">
-        <v>0.802</v>
+        <v>0.83</v>
       </c>
       <c r="I2" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>